<commit_message>
Domain + password update, percentage labels, mobile layout
- domain moves to turmericstudy.rs.org.pk (CNAME.pending, docs, footers)
- access password is now TS2026@RS; payload re-encrypted with it
- count-based bar charts label as "n (x%)" across 21 charts, with the
  share of the chart base also shown in the tooltip. Price, quantity and
  histogram charts keep raw units, where a share would be meaningless.
- twelve nav tabs were clipped on narrow screens; below 1000px they are
  replaced by a native section picker built from the same tab list
- phone layout reworked: horizontally scrolling filter row, tighter
  header ordering, taller chart canvases and earlier label wrapping so
  bars stay legible, responsive tables, funnel and matrix
- charts redraw when a rotation crosses the breakpoint
- payload URL now carries a build stamp; without it GitHub Pages caching
  served returning viewers the previous day's figures after an update
</commit_message>
<xml_diff>
--- a/instruments/turmeric_sampling_survey.xlsx
+++ b/instruments/turmeric_sampling_survey.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RS- Projects\Awareness Survey &amp; Turmeric Sampling\Turmeric Sampling\Instrument\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C02920-A587-4244-B05D-8D05CC833C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7087E86-8498-4E92-BAB8-A9196B8A7B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="627">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="627">
   <si>
     <t>type</t>
   </si>
@@ -3004,19 +3004,10 @@
     <t>Locality of Retail Market</t>
   </si>
   <si>
-    <t>select_one market_place</t>
-  </si>
-  <si>
     <t>wholesale_market</t>
   </si>
   <si>
-    <t>Wholesake Market Name</t>
-  </si>
-  <si>
     <t>city</t>
-  </si>
-  <si>
-    <t>market_place</t>
   </si>
   <si>
     <t>Jodia Bazaar</t>
@@ -3376,9 +3367,6 @@
     <t>Wahdat Colony Brewery Road</t>
   </si>
   <si>
-    <t>Mini Market Settelite Town</t>
-  </si>
-  <si>
     <t>Main Bazar Area Jinnah Road</t>
   </si>
   <si>
@@ -3523,69 +3511,12 @@
     <t>اس دکان پر کون کون سی قسم کی ہلدی دستیاب ہے؟</t>
   </si>
   <si>
-    <t>Phase 5 DHA Khadda market</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> PECHS/Tariq Road/Bahadurabad side</t>
-  </si>
-  <si>
     <t>Jodia bazar/Empres Market</t>
   </si>
   <si>
-    <t>Landhi Babar Market or Banaras Ali garh market orangi</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> autoban road nearby shops</t>
-  </si>
-  <si>
-    <t>faqir ka pir bazar</t>
-  </si>
-  <si>
-    <t>tower market retails side shops</t>
-  </si>
-  <si>
-    <t>Hayatabad shops</t>
-  </si>
-  <si>
-    <t>Board Bazar</t>
-  </si>
-  <si>
-    <t>Pipal mandi</t>
-  </si>
-  <si>
-    <t>Akbar Mandi wholesale and retail both shops are near by</t>
-  </si>
-  <si>
-    <t>ڈی ایچ اے فیز 5_کھڈا مارکیٹ</t>
-  </si>
-  <si>
-    <t>پی ای سی ایچ ایس_طارق روڈ_بہادر آباد</t>
-  </si>
-  <si>
     <t>جوڑیا بازار_ایمپریس مارکیٹ</t>
   </si>
   <si>
-    <t>لانڈھی بابر مارکیٹ یا بنارس علی گڑھ مارکیٹ اورنگی</t>
-  </si>
-  <si>
-    <t>آٹو بان روڈ کے نزدیک دکانیں</t>
-  </si>
-  <si>
-    <t>فقیر کا پیر بازار</t>
-  </si>
-  <si>
-    <t>ٹاور مارکیٹ ریٹیل سائیڈ دکانیں</t>
-  </si>
-  <si>
-    <t>حیات آباد کی دکانیں</t>
-  </si>
-  <si>
-    <t>بورڈ بازار</t>
-  </si>
-  <si>
-    <t>اکبر منڈی ہول سیل اور ریٹیل دونوں دکانیں نزدیک ہیں</t>
-  </si>
-  <si>
     <t>show_formatted</t>
   </si>
   <si>
@@ -3617,13 +3548,104 @@
   </si>
   <si>
     <t>selected(${shop_sample_type}, filter)</t>
+  </si>
+  <si>
+    <t>select_one wholesale_market</t>
+  </si>
+  <si>
+    <t>Wholesale Market Name</t>
+  </si>
+  <si>
+    <t>Mini Market Sattelite Town</t>
+  </si>
+  <si>
+    <t>Shalimar
+Akbar Mandi (wholesale and retail)</t>
+  </si>
+  <si>
+    <t>شالیمار
+اکبر منڈی (ہول سیل اور ریٹیل)</t>
+  </si>
+  <si>
+    <t>Sardar Ahmad Jan Colony
+Hayatabad shops</t>
+  </si>
+  <si>
+    <t>Khanza &amp; Bakhsho Pull
+Board Bazaar</t>
+  </si>
+  <si>
+    <t>Yousaf Abad
+Peepal Mandi</t>
+  </si>
+  <si>
+    <t>سردار احمد جان کالونی
+حیات آباد شاپس</t>
+  </si>
+  <si>
+    <t>خانزہ اینڈ بخشو پل
+بورڈ بازار</t>
+  </si>
+  <si>
+    <t>یوسف آباد
+پیپل منڈی</t>
+  </si>
+  <si>
+    <t>Liaqat Colony
+Tower Market</t>
+  </si>
+  <si>
+    <t>Hali Road
+Faqir ka Pir Bazaar</t>
+  </si>
+  <si>
+    <t>Latif Abad Unit # 06
+Autoban Road near shops</t>
+  </si>
+  <si>
+    <t>لطیف آباد یونٹ نمبر 06
+آٹو بان روڈ، دکانوں کے قریب</t>
+  </si>
+  <si>
+    <t>حالی روڈ
+فقیر کا پیر بازار</t>
+  </si>
+  <si>
+    <t>لیاقت کالونی
+ٹاور مارکیٹ</t>
+  </si>
+  <si>
+    <t>Shah Faisal Colony # 01_Sabzi Market
+Landhi Babar Market
+Banaras Aligarh Market Orangi</t>
+  </si>
+  <si>
+    <t>Gulshan e Iqbal_Block 10A
+PECHS/Tariq Road/Bahadurabad side</t>
+  </si>
+  <si>
+    <t>DHA Phase 5 Khadda Market
+Karachi Farmers' Market on weekends</t>
+  </si>
+  <si>
+    <t>ڈی ایچ اے فیز 5، کھڈا مارکیٹ
+کراچی فارمرز مارکیٹ، ہفتہ وار تعطیلات کے دن</t>
+  </si>
+  <si>
+    <t>گلشنِ اقبال، بلاک 10A
+پی ای سی ایچ ایس / طارق روڈ / بہادرآباد سائیڈ</t>
+  </si>
+  <si>
+    <t>شاہ فیصل کالونی نمبر 01، سبزی مارکیٹ
+لانڈھی، بابر مارکیٹ
+بنارس علی گڑھ مارکیٹ، اورنگی</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3722,13 +3744,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Arabic Typesetting"/>
-      <family val="4"/>
-      <charset val="178"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -3792,7 +3807,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -3970,17 +3985,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -4098,14 +4102,8 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4130,6 +4128,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4651,7 +4655,7 @@
       <c r="O1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="44" t="s">
+      <c r="P1" s="43" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="7" t="s">
@@ -5220,7 +5224,7 @@
         <v>369</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="8"/>
@@ -5263,7 +5267,7 @@
       <c r="M19" s="9"/>
       <c r="N19" s="8"/>
       <c r="O19" s="9" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="P19" s="8"/>
       <c r="Q19" s="8"/>
@@ -5286,7 +5290,7 @@
         <v>424</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="8"/>
@@ -5313,7 +5317,7 @@
     </row>
     <row r="21" spans="1:24" ht="39">
       <c r="A21" s="9" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="B21" s="9" t="s">
         <v>425</v>
@@ -5322,7 +5326,7 @@
         <v>427</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="8"/>
@@ -5330,7 +5334,7 @@
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
       <c r="J21" s="9" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
@@ -5344,7 +5348,7 @@
       <c r="R21" s="8"/>
       <c r="S21" s="8"/>
       <c r="T21" s="8" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="U21" s="8"/>
       <c r="V21" s="8"/>
@@ -5353,16 +5357,16 @@
     </row>
     <row r="22" spans="1:24" ht="39">
       <c r="A22" s="9" t="s">
+        <v>604</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>428</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>429</v>
-      </c>
       <c r="C22" s="9" t="s">
-        <v>430</v>
+        <v>605</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="E22" s="9"/>
       <c r="F22" s="8"/>
@@ -5370,7 +5374,7 @@
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
@@ -5384,7 +5388,7 @@
       <c r="R22" s="8"/>
       <c r="S22" s="8"/>
       <c r="T22" s="8" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="U22" s="8"/>
       <c r="V22" s="8"/>
@@ -5399,10 +5403,10 @@
         <v>364</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="E23" s="9"/>
       <c r="F23" s="8"/>
@@ -5432,13 +5436,13 @@
         <v>389</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>617</v>
+        <v>594</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="8"/>
@@ -5468,16 +5472,16 @@
         <v>389</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>618</v>
+        <v>595</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>619</v>
+        <v>596</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>620</v>
+        <v>597</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>621</v>
+        <v>598</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="9"/>
@@ -5496,7 +5500,7 @@
       <c r="R25" s="8"/>
       <c r="S25" s="8"/>
       <c r="T25" s="8" t="s">
-        <v>626</v>
+        <v>603</v>
       </c>
       <c r="U25" s="8"/>
       <c r="V25" s="8"/>
@@ -5514,7 +5518,7 @@
         <v>370</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="8"/>
@@ -5523,9 +5527,7 @@
       <c r="I26" s="9"/>
       <c r="J26" s="9"/>
       <c r="K26" s="8"/>
-      <c r="L26" s="8" t="s">
-        <v>47</v>
-      </c>
+      <c r="L26" s="8"/>
       <c r="M26" s="9"/>
       <c r="N26" s="8"/>
       <c r="O26" s="9"/>
@@ -5550,7 +5552,7 @@
         <v>387</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="E27" s="9"/>
       <c r="F27" s="8"/>
@@ -5586,7 +5588,7 @@
         <v>403</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="E28" s="9"/>
       <c r="F28" s="8"/>
@@ -5600,7 +5602,7 @@
       <c r="N28" s="8"/>
       <c r="O28" s="9"/>
       <c r="P28" s="8" t="s">
-        <v>622</v>
+        <v>599</v>
       </c>
       <c r="Q28" s="8"/>
       <c r="R28" s="8"/>
@@ -5631,7 +5633,7 @@
       <c r="M29" s="9"/>
       <c r="N29" s="8"/>
       <c r="O29" s="9" t="s">
-        <v>623</v>
+        <v>600</v>
       </c>
       <c r="P29" s="8"/>
       <c r="Q29" s="8"/>
@@ -5663,7 +5665,7 @@
       <c r="M30" s="9"/>
       <c r="N30" s="8"/>
       <c r="O30" s="9" t="s">
-        <v>624</v>
+        <v>601</v>
       </c>
       <c r="P30" s="8"/>
       <c r="Q30" s="8"/>
@@ -5686,7 +5688,7 @@
         <v>407</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="E31" s="9"/>
       <c r="F31" s="8"/>
@@ -5720,7 +5722,7 @@
         <v>408</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="E32" s="9"/>
       <c r="F32" s="8"/>
@@ -5760,7 +5762,7 @@
         <v>411</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="E33" s="9"/>
       <c r="F33" s="8"/>
@@ -5796,7 +5798,7 @@
         <v>413</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="E34" s="9"/>
       <c r="F34" s="8"/>
@@ -5829,15 +5831,15 @@
         <v>396</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="8"/>
       <c r="G35" s="9" t="s">
-        <v>616</v>
+        <v>593</v>
       </c>
       <c r="H35" s="9" t="s">
         <v>409</v>
@@ -5871,10 +5873,10 @@
         <v>397</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="8"/>
@@ -5914,7 +5916,7 @@
         <v>416</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="E37" s="9"/>
       <c r="F37" s="8"/>
@@ -5948,7 +5950,7 @@
         <v>400</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="E38" s="9"/>
       <c r="F38" s="8"/>
@@ -5998,7 +6000,7 @@
         <v>66</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>625</v>
+        <v>602</v>
       </c>
       <c r="L41" s="9" t="s">
         <v>47</v>
@@ -6018,6 +6020,7 @@
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="10" style="5" customWidth="1"/>
     <col min="3" max="4" width="54.85546875" style="5" customWidth="1"/>
+    <col min="6" max="7" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -6036,10 +6039,10 @@
       <c r="E1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="G1" s="45" t="s">
+      <c r="F1" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="G1" s="55" t="s">
         <v>70</v>
       </c>
     </row>
@@ -6051,13 +6054,14 @@
         <v>71</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
@@ -6067,13 +6071,14 @@
         <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
@@ -6083,13 +6088,14 @@
         <v>73</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
@@ -6099,13 +6105,14 @@
         <v>74</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
@@ -6115,13 +6122,14 @@
         <v>75</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
@@ -6131,13 +6139,14 @@
         <v>76</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="2" t="s">
@@ -6147,13 +6156,14 @@
         <v>353</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="2" t="s">
@@ -6163,13 +6173,14 @@
         <v>354</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="2" t="s">
@@ -6179,13 +6190,14 @@
         <v>355</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
@@ -6195,13 +6207,14 @@
         <v>356</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="2" t="s">
@@ -6211,111 +6224,118 @@
         <v>357</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6">
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" s="2" t="s">
         <v>53</v>
       </c>
@@ -6323,15 +6343,16 @@
         <v>777</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" s="2" t="s">
         <v>85</v>
       </c>
@@ -6345,9 +6366,10 @@
         <v>86</v>
       </c>
       <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" s="2" t="s">
         <v>85</v>
       </c>
@@ -6361,9 +6383,10 @@
         <v>87</v>
       </c>
       <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" s="2" t="s">
         <v>85</v>
       </c>
@@ -6377,9 +6400,10 @@
         <v>88</v>
       </c>
       <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" s="2" t="s">
         <v>85</v>
       </c>
@@ -6393,9 +6417,10 @@
         <v>89</v>
       </c>
       <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" s="2" t="s">
         <v>85</v>
       </c>
@@ -6409,9 +6434,10 @@
         <v>90</v>
       </c>
       <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" s="2" t="s">
         <v>85</v>
       </c>
@@ -6425,9 +6451,10 @@
         <v>91</v>
       </c>
       <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" s="2" t="s">
         <v>85</v>
       </c>
@@ -6441,9 +6468,10 @@
         <v>92</v>
       </c>
       <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" s="2" t="s">
         <v>85</v>
       </c>
@@ -6457,9 +6485,10 @@
         <v>93</v>
       </c>
       <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" s="2" t="s">
         <v>85</v>
       </c>
@@ -6473,9 +6502,10 @@
         <v>95</v>
       </c>
       <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" s="2" t="s">
         <v>85</v>
       </c>
@@ -6489,9 +6519,10 @@
         <v>97</v>
       </c>
       <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" s="2" t="s">
         <v>371</v>
       </c>
@@ -6502,12 +6533,13 @@
         <v>372</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" s="2" t="s">
         <v>371</v>
       </c>
@@ -6518,12 +6550,13 @@
         <v>426</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-    </row>
-    <row r="32" spans="1:6">
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" s="2" t="s">
         <v>373</v>
       </c>
@@ -6534,10 +6567,11 @@
         <v>374</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="2" t="s">
@@ -6550,10 +6584,11 @@
         <v>375</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="2" t="s">
@@ -6566,10 +6601,11 @@
         <v>376</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="2" t="s">
@@ -6582,10 +6618,11 @@
         <v>377</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="2" t="s">
@@ -6598,10 +6635,11 @@
         <v>378</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="2" t="s">
@@ -6614,10 +6652,11 @@
         <v>379</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="2" t="s">
@@ -6630,10 +6669,11 @@
         <v>380</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="2" t="s">
@@ -6646,10 +6686,11 @@
         <v>381</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="2" t="s">
@@ -6662,10 +6703,11 @@
         <v>382</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="2" t="s">
@@ -6678,10 +6720,11 @@
         <v>383</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" s="2" t="s">
@@ -6691,14 +6734,14 @@
         <v>1</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42">
+      <c r="F42" s="4"/>
+      <c r="G42" s="4">
         <v>1</v>
       </c>
     </row>
@@ -6710,14 +6753,14 @@
         <v>2</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43">
+      <c r="F43" s="4"/>
+      <c r="G43" s="4">
         <v>2</v>
       </c>
     </row>
@@ -6729,14 +6772,14 @@
         <v>3</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44">
+      <c r="F44" s="4"/>
+      <c r="G44" s="4">
         <v>3</v>
       </c>
     </row>
@@ -6748,14 +6791,14 @@
         <v>4</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45">
+      <c r="F45" s="4"/>
+      <c r="G45" s="4">
         <v>4</v>
       </c>
     </row>
@@ -6770,10 +6813,11 @@
         <v>392</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="2" t="s">
@@ -6786,10 +6830,11 @@
         <v>393</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="2" t="s">
@@ -6802,12 +6847,13 @@
         <v>394</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-    </row>
-    <row r="49" spans="1:6">
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" s="2" t="s">
         <v>391</v>
       </c>
@@ -6818,12 +6864,13 @@
         <v>395</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-    </row>
-    <row r="50" spans="1:6">
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" s="2" t="s">
         <v>420</v>
       </c>
@@ -6834,12 +6881,13 @@
         <v>421</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-    </row>
-    <row r="51" spans="1:6">
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+    </row>
+    <row r="51" spans="1:7">
       <c r="A51" s="2" t="s">
         <v>420</v>
       </c>
@@ -6850,12 +6898,13 @@
         <v>422</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-    </row>
-    <row r="52" spans="1:6">
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" s="2" t="s">
         <v>420</v>
       </c>
@@ -6866,964 +6915,1018 @@
         <v>423</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-    </row>
-    <row r="53" spans="1:6">
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B53" s="4">
         <v>1</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="E53" s="2"/>
-      <c r="F53" s="2">
+      <c r="F53" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:6">
+      <c r="G53" s="4"/>
+    </row>
+    <row r="54" spans="1:7">
       <c r="A54" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B54" s="4">
         <v>2</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="E54" s="2"/>
-      <c r="F54" s="2">
+      <c r="F54" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:6">
+      <c r="G54" s="4"/>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B55" s="4">
         <v>3</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="E55" s="2"/>
-      <c r="F55" s="2">
+      <c r="F55" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="56" spans="1:6">
+      <c r="G55" s="4"/>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B56" s="4">
         <v>4</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="E56" s="2"/>
-      <c r="F56" s="2">
+      <c r="F56" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="57" spans="1:6">
+      <c r="G56" s="4"/>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B57" s="4">
         <v>5</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="E57" s="2"/>
-      <c r="F57" s="2">
+      <c r="F57" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="58" spans="1:6">
+      <c r="G57" s="4"/>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B58" s="4">
         <v>6</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="E58" s="2"/>
-      <c r="F58" s="2">
+      <c r="F58" s="4">
         <v>7</v>
       </c>
-    </row>
-    <row r="59" spans="1:6">
+      <c r="G58" s="4"/>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B59" s="4">
         <v>7</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="E59" s="2"/>
-      <c r="F59" s="2">
+      <c r="F59" s="4">
         <v>8</v>
       </c>
-    </row>
-    <row r="60" spans="1:6">
+      <c r="G59" s="4"/>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B60" s="4">
         <v>8</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="E60" s="2"/>
-      <c r="F60" s="2">
+      <c r="F60" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="61" spans="1:6">
+      <c r="G60" s="4"/>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B61" s="4">
         <v>9</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="E61" s="2"/>
-      <c r="F61" s="2">
+      <c r="F61" s="4">
         <v>10</v>
       </c>
-    </row>
-    <row r="62" spans="1:6">
+      <c r="G61" s="4"/>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B62" s="4">
         <v>10</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="E62" s="2"/>
-      <c r="F62" s="2">
+      <c r="F62" s="4">
         <v>9</v>
       </c>
-    </row>
-    <row r="63" spans="1:6">
+      <c r="G62" s="4"/>
+    </row>
+    <row r="63" spans="1:7">
       <c r="A63" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B63" s="4">
         <v>11</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="E63" s="2"/>
-      <c r="F63" s="2">
+      <c r="F63" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="64" spans="1:6">
+      <c r="G63" s="4"/>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B64" s="4">
         <v>12</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="E64" s="2"/>
-      <c r="F64" s="2">
+      <c r="F64" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="65" spans="1:6">
+      <c r="G64" s="4"/>
+    </row>
+    <row r="65" spans="1:7">
       <c r="A65" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B65" s="4">
         <v>13</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="E65" s="2"/>
-      <c r="F65" s="2">
+      <c r="F65" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" ht="19.5">
+      <c r="G65" s="4"/>
+    </row>
+    <row r="66" spans="1:7" ht="30">
       <c r="A66" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B66" s="4">
         <v>1</v>
       </c>
-      <c r="C66" s="4" t="s">
-        <v>595</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>606</v>
+      <c r="C66" s="56" t="s">
+        <v>623</v>
+      </c>
+      <c r="D66" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="E66" s="2"/>
-      <c r="F66" s="43">
+      <c r="F66" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" ht="19.5">
+      <c r="G66" s="4"/>
+    </row>
+    <row r="67" spans="1:7" ht="30">
       <c r="A67" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B67" s="4">
         <v>2</v>
       </c>
-      <c r="C67" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>607</v>
+      <c r="C67" s="56" t="s">
+        <v>622</v>
+      </c>
+      <c r="D67" s="56" t="s">
+        <v>625</v>
       </c>
       <c r="E67" s="2"/>
-      <c r="F67" s="43">
+      <c r="F67" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" ht="19.5">
+      <c r="G67" s="4"/>
+    </row>
+    <row r="68" spans="1:7">
       <c r="A68" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B68" s="4">
         <v>3</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>597</v>
+        <v>591</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>608</v>
+        <v>592</v>
       </c>
       <c r="E68" s="2"/>
-      <c r="F68" s="43">
+      <c r="F68" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" ht="19.5">
+      <c r="G68" s="4"/>
+    </row>
+    <row r="69" spans="1:7" ht="45">
       <c r="A69" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B69" s="4">
         <v>4</v>
       </c>
-      <c r="C69" s="4" t="s">
-        <v>598</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>609</v>
+      <c r="C69" s="56" t="s">
+        <v>621</v>
+      </c>
+      <c r="D69" s="56" t="s">
+        <v>626</v>
       </c>
       <c r="E69" s="2"/>
-      <c r="F69" s="43">
+      <c r="F69" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" ht="19.5">
+      <c r="G69" s="4"/>
+    </row>
+    <row r="70" spans="1:7" ht="30">
       <c r="A70" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B70" s="4">
         <v>5</v>
       </c>
-      <c r="C70" s="4" t="s">
-        <v>599</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>610</v>
+      <c r="C70" s="56" t="s">
+        <v>617</v>
+      </c>
+      <c r="D70" s="56" t="s">
+        <v>618</v>
       </c>
       <c r="E70" s="2"/>
-      <c r="F70" s="43">
+      <c r="F70" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" ht="19.5">
+      <c r="G70" s="4"/>
+    </row>
+    <row r="71" spans="1:7">
       <c r="A71" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B71" s="4">
         <v>6</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="E71" s="2"/>
-      <c r="F71" s="43">
+      <c r="F71" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" ht="19.5">
+      <c r="G71" s="4"/>
+    </row>
+    <row r="72" spans="1:7" ht="30">
       <c r="A72" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B72" s="4">
         <v>7</v>
       </c>
-      <c r="C72" s="4" t="s">
-        <v>600</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>611</v>
+      <c r="C72" s="56" t="s">
+        <v>616</v>
+      </c>
+      <c r="D72" s="56" t="s">
+        <v>619</v>
       </c>
       <c r="E72" s="2"/>
-      <c r="F72" s="43">
+      <c r="F72" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" ht="19.5">
+      <c r="G72" s="4"/>
+    </row>
+    <row r="73" spans="1:7" ht="30">
       <c r="A73" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B73" s="4">
         <v>8</v>
       </c>
-      <c r="C73" s="4" t="s">
-        <v>601</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>612</v>
+      <c r="C73" s="56" t="s">
+        <v>615</v>
+      </c>
+      <c r="D73" s="56" t="s">
+        <v>620</v>
       </c>
       <c r="E73" s="2"/>
-      <c r="F73" s="43">
+      <c r="F73" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" ht="19.5">
+      <c r="G73" s="4"/>
+    </row>
+    <row r="74" spans="1:7">
       <c r="A74" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B74" s="4">
         <v>9</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="E74" s="2"/>
-      <c r="F74" s="43">
+      <c r="F74" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" ht="19.5">
+      <c r="G74" s="4"/>
+    </row>
+    <row r="75" spans="1:7" ht="30">
       <c r="A75" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B75" s="4">
         <v>10</v>
       </c>
-      <c r="C75" s="4" t="s">
-        <v>602</v>
-      </c>
-      <c r="D75" s="4" t="s">
-        <v>613</v>
+      <c r="C75" s="56" t="s">
+        <v>609</v>
+      </c>
+      <c r="D75" s="56" t="s">
+        <v>612</v>
       </c>
       <c r="E75" s="2"/>
-      <c r="F75" s="43">
+      <c r="F75" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" ht="19.5">
+      <c r="G75" s="4"/>
+    </row>
+    <row r="76" spans="1:7" ht="30">
       <c r="A76" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B76" s="4">
         <v>11</v>
       </c>
-      <c r="C76" s="4" t="s">
-        <v>603</v>
-      </c>
-      <c r="D76" s="4" t="s">
-        <v>614</v>
+      <c r="C76" s="56" t="s">
+        <v>610</v>
+      </c>
+      <c r="D76" s="56" t="s">
+        <v>613</v>
       </c>
       <c r="E76" s="2"/>
-      <c r="F76" s="43">
+      <c r="F76" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" ht="19.5">
+      <c r="G76" s="4"/>
+    </row>
+    <row r="77" spans="1:7" ht="30">
       <c r="A77" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B77" s="4">
         <v>12</v>
       </c>
-      <c r="C77" s="4" t="s">
-        <v>604</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>512</v>
+      <c r="C77" s="56" t="s">
+        <v>611</v>
+      </c>
+      <c r="D77" s="56" t="s">
+        <v>614</v>
       </c>
       <c r="E77" s="2"/>
-      <c r="F77" s="43">
+      <c r="F77" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" ht="19.5">
+      <c r="G77" s="4"/>
+    </row>
+    <row r="78" spans="1:7">
       <c r="A78" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B78" s="4">
         <v>13</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E78" s="2"/>
-      <c r="F78" s="43">
+      <c r="F78" s="4">
         <v>7</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" ht="19.5">
+      <c r="G78" s="4"/>
+    </row>
+    <row r="79" spans="1:7">
       <c r="A79" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B79" s="4">
         <v>14</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="E79" s="2"/>
-      <c r="F79" s="43">
+      <c r="F79" s="4">
         <v>7</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" ht="19.5">
+      <c r="G79" s="4"/>
+    </row>
+    <row r="80" spans="1:7">
       <c r="A80" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B80" s="4">
         <v>15</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="E80" s="2"/>
-      <c r="F80" s="43">
+      <c r="F80" s="4">
         <v>7</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" ht="19.5">
+      <c r="G80" s="4"/>
+    </row>
+    <row r="81" spans="1:7" ht="30">
       <c r="A81" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B81" s="4">
         <v>16</v>
       </c>
-      <c r="C81" s="4" t="s">
-        <v>605</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>615</v>
+      <c r="C81" s="56" t="s">
+        <v>607</v>
+      </c>
+      <c r="D81" s="56" t="s">
+        <v>608</v>
       </c>
       <c r="E81" s="2"/>
-      <c r="F81" s="43">
+      <c r="F81" s="4">
         <v>7</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" ht="19.5">
+      <c r="G81" s="4"/>
+    </row>
+    <row r="82" spans="1:7">
       <c r="A82" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B82" s="4">
         <v>17</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="E82" s="2"/>
-      <c r="F82" s="43">
+      <c r="F82" s="4">
         <v>10</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" ht="19.5">
+      <c r="G82" s="4"/>
+    </row>
+    <row r="83" spans="1:7">
       <c r="A83" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B83" s="4">
         <v>18</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="E83" s="2"/>
-      <c r="F83" s="43">
+      <c r="F83" s="4">
         <v>10</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" ht="19.5">
+      <c r="G83" s="4"/>
+    </row>
+    <row r="84" spans="1:7">
       <c r="A84" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B84" s="4">
         <v>19</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="E84" s="2"/>
-      <c r="F84" s="43">
+      <c r="F84" s="4">
         <v>10</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" ht="19.5">
+      <c r="G84" s="4"/>
+    </row>
+    <row r="85" spans="1:7">
       <c r="A85" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B85" s="4">
         <v>20</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="E85" s="2"/>
-      <c r="F85" s="43">
+      <c r="F85" s="4">
         <v>10</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" ht="19.5">
+      <c r="G85" s="4"/>
+    </row>
+    <row r="86" spans="1:7">
       <c r="A86" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B86" s="4">
         <v>21</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
       <c r="E86" s="2"/>
-      <c r="F86" s="43">
+      <c r="F86" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" ht="19.5">
+      <c r="G86" s="4"/>
+    </row>
+    <row r="87" spans="1:7">
       <c r="A87" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B87" s="4">
         <v>22</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="E87" s="2"/>
-      <c r="F87" s="43">
+      <c r="F87" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" ht="19.5">
+      <c r="G87" s="4"/>
+    </row>
+    <row r="88" spans="1:7">
       <c r="A88" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B88" s="4">
         <v>23</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>546</v>
+        <v>606</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="E88" s="2"/>
-      <c r="F88" s="43">
+      <c r="F88" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" ht="19.5">
+      <c r="G88" s="4"/>
+    </row>
+    <row r="89" spans="1:7">
       <c r="A89" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B89" s="4">
         <v>24</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="E89" s="2"/>
-      <c r="F89" s="43">
+      <c r="F89" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" ht="19.5">
+      <c r="G89" s="4"/>
+    </row>
+    <row r="90" spans="1:7">
       <c r="A90" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B90" s="4">
         <v>25</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>577</v>
+        <v>573</v>
       </c>
       <c r="E90" s="2"/>
-      <c r="F90" s="43">
+      <c r="F90" s="4">
         <v>9</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" ht="19.5">
+      <c r="G90" s="4"/>
+    </row>
+    <row r="91" spans="1:7">
       <c r="A91" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B91" s="4">
         <v>26</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="E91" s="2"/>
-      <c r="F91" s="43">
+      <c r="F91" s="4">
         <v>9</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" ht="19.5">
+      <c r="G91" s="4"/>
+    </row>
+    <row r="92" spans="1:7">
       <c r="A92" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B92" s="4">
         <v>27</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="E92" s="2"/>
-      <c r="F92" s="43">
+      <c r="F92" s="4">
         <v>9</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" ht="19.5">
+      <c r="G92" s="4"/>
+    </row>
+    <row r="93" spans="1:7">
       <c r="A93" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B93" s="4">
         <v>28</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="E93" s="2"/>
-      <c r="F93" s="43">
+      <c r="F93" s="4">
         <v>9</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" ht="19.5">
+      <c r="G93" s="4"/>
+    </row>
+    <row r="94" spans="1:7">
       <c r="A94" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B94" s="4">
         <v>29</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="E94" s="2"/>
-      <c r="F94" s="43">
+      <c r="F94" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" ht="19.5">
+      <c r="G94" s="4"/>
+    </row>
+    <row r="95" spans="1:7">
       <c r="A95" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B95" s="4">
         <v>30</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="E95" s="2"/>
-      <c r="F95" s="43">
+      <c r="F95" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" ht="19.5">
+      <c r="G95" s="4"/>
+    </row>
+    <row r="96" spans="1:7">
       <c r="A96" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B96" s="4">
         <v>31</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="E96" s="2"/>
-      <c r="F96" s="43">
+      <c r="F96" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" ht="19.5">
+      <c r="G96" s="4"/>
+    </row>
+    <row r="97" spans="1:7">
       <c r="A97" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B97" s="4">
         <v>32</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="E97" s="2"/>
-      <c r="F97" s="43">
+      <c r="F97" s="4">
         <v>4</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" ht="19.5">
+      <c r="G97" s="4"/>
+    </row>
+    <row r="98" spans="1:7">
       <c r="A98" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B98" s="4">
         <v>33</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="E98" s="2"/>
-      <c r="F98" s="43">
+      <c r="F98" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" ht="19.5">
+      <c r="G98" s="4"/>
+    </row>
+    <row r="99" spans="1:7">
       <c r="A99" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B99" s="4">
         <v>34</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="E99" s="2"/>
-      <c r="F99" s="43">
+      <c r="F99" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" ht="19.5">
+      <c r="G99" s="4"/>
+    </row>
+    <row r="100" spans="1:7">
       <c r="A100" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B100" s="4">
         <v>35</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="E100" s="2"/>
-      <c r="F100" s="43">
+      <c r="F100" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" ht="19.5">
+      <c r="G100" s="4"/>
+    </row>
+    <row r="101" spans="1:7">
       <c r="A101" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B101" s="4">
         <v>36</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="E101" s="2"/>
-      <c r="F101" s="43">
+      <c r="F101" s="4">
         <v>5</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" ht="19.5">
+      <c r="G101" s="4"/>
+    </row>
+    <row r="102" spans="1:7">
       <c r="A102" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B102" s="4">
         <v>37</v>
       </c>
       <c r="C102" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="E102" s="2"/>
+      <c r="F102" s="4">
+        <v>8</v>
+      </c>
+      <c r="G102" s="4"/>
+    </row>
+    <row r="103" spans="1:7">
+      <c r="A103" s="2" t="s">
         <v>560</v>
-      </c>
-      <c r="D102" s="4" t="s">
-        <v>589</v>
-      </c>
-      <c r="E102" s="2"/>
-      <c r="F102" s="43">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" ht="19.5">
-      <c r="A103" s="2" t="s">
-        <v>564</v>
       </c>
       <c r="B103" s="4">
         <v>38</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="E103" s="2"/>
-      <c r="F103" s="43">
+      <c r="F103" s="4">
         <v>8</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" ht="19.5">
+      <c r="G103" s="4"/>
+    </row>
+    <row r="104" spans="1:7">
       <c r="A104" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B104" s="4">
         <v>39</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="E104" s="2"/>
-      <c r="F104" s="43">
+      <c r="F104" s="4">
         <v>8</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" ht="19.5">
+      <c r="G104" s="4"/>
+    </row>
+    <row r="105" spans="1:7">
       <c r="A105" s="2" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="B105" s="4">
         <v>40</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E105" s="2"/>
-      <c r="F105" s="43">
+      <c r="F105" s="4">
         <v>8</v>
       </c>
+      <c r="G105" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
@@ -7883,7 +7986,7 @@
       </c>
       <c r="C2" t="str">
         <f ca="1">TEXT(YEAR(NOW())-2000,"00")&amp;TEXT(MONTH(NOW()),"00")&amp;TEXT(DAY(NOW()),"00")&amp;TEXT(HOUR(NOW()),"00")&amp;TEXT(MINUTE(NOW()),"00")</f>
-        <v>2608061815</v>
+        <v>2608101435</v>
       </c>
       <c r="F2" t="s">
         <v>104</v>
@@ -7904,20 +8007,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="44" t="s">
         <v>307</v>
       </c>
-      <c r="B1" s="47"/>
+      <c r="B1" s="45"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="49"/>
+      <c r="A2" s="46"/>
+      <c r="B2" s="47"/>
     </row>
     <row r="3" spans="1:17" ht="99" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="48" t="s">
         <v>312</v>
       </c>
-      <c r="B3" s="51"/>
+      <c r="B3" s="49"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="5" spans="1:17" ht="18" customHeight="1">
@@ -8999,22 +9102,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="15.75">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="47"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="49"/>
+      <c r="A2" s="46"/>
+      <c r="B2" s="47"/>
       <c r="C2" s="18"/>
     </row>
     <row r="3" spans="1:30" ht="96.75" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="48" t="s">
         <v>320</v>
       </c>
-      <c r="B3" s="51"/>
+      <c r="B3" s="49"/>
       <c r="C3" s="18"/>
     </row>
     <row r="4" spans="1:30" ht="15.75" customHeight="1">
@@ -9208,10 +9311,10 @@
       <c r="C7" s="18"/>
     </row>
     <row r="8" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="50" t="s">
         <v>347</v>
       </c>
-      <c r="B8" s="53"/>
+      <c r="B8" s="51"/>
       <c r="C8" s="22"/>
       <c r="D8" s="23"/>
       <c r="E8" s="23"/>
@@ -11732,10 +11835,10 @@
       <c r="C75" s="18"/>
     </row>
     <row r="76" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A76" s="54" t="s">
+      <c r="A76" s="52" t="s">
         <v>199</v>
       </c>
-      <c r="B76" s="53"/>
+      <c r="B76" s="51"/>
       <c r="C76" s="28"/>
       <c r="D76" s="29"/>
       <c r="E76" s="30"/>
@@ -13294,28 +13397,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" customHeight="1">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="53" t="s">
         <v>309</v>
       </c>
-      <c r="B1" s="56"/>
+      <c r="B1" s="54"/>
       <c r="C1" s="37"/>
       <c r="D1" s="37"/>
       <c r="E1" s="37"/>
       <c r="F1" s="37"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1">
-      <c r="A2" s="48"/>
-      <c r="B2" s="49"/>
+      <c r="A2" s="46"/>
+      <c r="B2" s="47"/>
       <c r="C2" s="37"/>
       <c r="D2" s="37"/>
       <c r="E2" s="37"/>
       <c r="F2" s="37"/>
     </row>
     <row r="3" spans="1:16" ht="54.75" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="48" t="s">
         <v>310</v>
       </c>
-      <c r="B3" s="51"/>
+      <c r="B3" s="49"/>
       <c r="C3" s="37"/>
       <c r="D3" s="37"/>
       <c r="E3" s="37"/>

</xml_diff>

<commit_message>
Ship the app.js half of the eleven-panel rebuild
The last data update pushed the new index.html (Field Ops retired, new
charts added) but left assets/app.js in the working tree, so the live
page carried eleven canvases nothing ever drew — ovCumAw, ovCumTs,
smRootDisplay, smBasisType, ldCity, ldSplit, mapCityStack, mdCity,
prBox, prMkt, rtTopBottom all rendered blank.

Also ships the matching theme.css, the whole_root_display field in the
builder, and the demo generator fixes for codes that had no label.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/instruments/turmeric_sampling_survey.xlsx
+++ b/instruments/turmeric_sampling_survey.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RS- Projects\Awareness Survey &amp; Turmeric Sampling\Turmeric Sampling\Instrument\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7087E86-8498-4E92-BAB8-A9196B8A7B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63990283-5605-42FE-A762-C9FE4D73717C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="627">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="638">
   <si>
     <t>type</t>
   </si>
@@ -3639,6 +3639,39 @@
     <t>شاہ فیصل کالونی نمبر 01، سبزی مارکیٹ
 لانڈھی، بابر مارکیٹ
 بنارس علی گڑھ مارکیٹ، اورنگی</t>
+  </si>
+  <si>
+    <t>root_display</t>
+  </si>
+  <si>
+    <t>Openly displayed (visible to customers)</t>
+  </si>
+  <si>
+    <t>کھلے عام نمائش پر (گاہکوں کو نظر آنے والی جگہ)</t>
+  </si>
+  <si>
+    <t>Not displayed – brought from back/inside upon asking</t>
+  </si>
+  <si>
+    <t>نمائش پر نہیں – پوچھنے پر اندر/پیچھے سے لا کر دکھائی</t>
+  </si>
+  <si>
+    <t>select_one root_display</t>
+  </si>
+  <si>
+    <t>whole_root_display</t>
+  </si>
+  <si>
+    <t>Were the whole dried roots openly displayed, or brought from the back/inside the store upon asking?</t>
+  </si>
+  <si>
+    <t>کیا ثابت خشک ہلدی کی جڑیں کھلے عام نمائش پر تھیں، یا پوچھنے پر دکان کے اندر/پیچھے سے لائی گئیں؟</t>
+  </si>
+  <si>
+    <t>Enumerator observation – for whole dried roots only</t>
+  </si>
+  <si>
+    <t>selected(${shop_sample_type}, '1')</t>
   </si>
 </sst>
 </file>
@@ -3990,7 +4023,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -4105,6 +4138,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4128,12 +4167,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4558,7 +4596,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="5">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="5">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -4580,33 +4618,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X41"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:X42"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="79.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="82.42578125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" customWidth="1"/>
-    <col min="7" max="7" width="28.42578125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="36.5703125" style="6" customWidth="1"/>
-    <col min="9" max="9" width="22.5703125" style="6" customWidth="1"/>
-    <col min="10" max="10" width="58.28515625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" customWidth="1"/>
-    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.140625" style="6" customWidth="1"/>
-    <col min="14" max="14" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="87.42578125" style="6" customWidth="1"/>
-    <col min="16" max="16" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.26953125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="23.453125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="79.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="82.453125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" customWidth="1"/>
+    <col min="7" max="7" width="28.453125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="36.54296875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="22.54296875" style="6" customWidth="1"/>
+    <col min="10" max="10" width="58.26953125" style="6" customWidth="1"/>
+    <col min="11" max="11" width="10.7265625" customWidth="1"/>
+    <col min="12" max="12" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.1796875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="87.453125" style="6" customWidth="1"/>
+    <col min="16" max="16" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="27.75" customHeight="1">
@@ -5541,7 +5579,7 @@
       <c r="W26" s="8"/>
       <c r="X26" s="8"/>
     </row>
-    <row r="27" spans="1:24" ht="39">
+    <row r="27" spans="1:24" ht="19.5">
       <c r="A27" s="9" t="s">
         <v>385</v>
       </c>
@@ -5613,7 +5651,7 @@
       <c r="W28" s="8"/>
       <c r="X28" s="8"/>
     </row>
-    <row r="29" spans="1:24" ht="39">
+    <row r="29" spans="1:24" ht="19.5">
       <c r="A29" s="9" t="s">
         <v>35</v>
       </c>
@@ -5711,7 +5749,7 @@
       <c r="W31" s="8"/>
       <c r="X31" s="8"/>
     </row>
-    <row r="32" spans="1:24" ht="58.5">
+    <row r="32" spans="1:24" ht="39">
       <c r="A32" s="9" t="s">
         <v>62</v>
       </c>
@@ -5989,23 +6027,47 @@
       <c r="B40" s="42"/>
       <c r="P40" s="8"/>
     </row>
-    <row r="41" spans="1:24" s="9" customFormat="1" ht="39">
-      <c r="A41" s="9" t="s">
+    <row r="41" spans="1:24" s="57" customFormat="1" ht="136.5">
+      <c r="A41" s="57" t="s">
+        <v>632</v>
+      </c>
+      <c r="B41" s="57" t="s">
+        <v>633</v>
+      </c>
+      <c r="C41" s="57" t="s">
+        <v>634</v>
+      </c>
+      <c r="D41" s="57" t="s">
+        <v>635</v>
+      </c>
+      <c r="E41" s="57" t="s">
+        <v>636</v>
+      </c>
+      <c r="J41" s="57" t="s">
+        <v>637</v>
+      </c>
+      <c r="L41" s="57" t="s">
+        <v>47</v>
+      </c>
+      <c r="P41" s="58"/>
+    </row>
+    <row r="42" spans="1:24" s="9" customFormat="1" ht="39">
+      <c r="A42" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="B42" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C42" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="D42" s="9" t="s">
         <v>602</v>
       </c>
-      <c r="L41" s="9" t="s">
+      <c r="L42" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="P41" s="8"/>
+      <c r="P42" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6014,13 +6076,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G105"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:G107"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="10" style="5" customWidth="1"/>
-    <col min="3" max="4" width="54.85546875" style="5" customWidth="1"/>
-    <col min="6" max="7" width="9.140625" style="5"/>
+    <col min="3" max="4" width="54.81640625" style="5" customWidth="1"/>
+    <col min="6" max="7" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -6042,7 +6104,7 @@
       <c r="F1" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="G1" s="55" t="s">
+      <c r="G1" s="44" t="s">
         <v>70</v>
       </c>
     </row>
@@ -7168,17 +7230,17 @@
       </c>
       <c r="G65" s="4"/>
     </row>
-    <row r="66" spans="1:7" ht="30">
+    <row r="66" spans="1:7" ht="29">
       <c r="A66" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B66" s="4">
         <v>1</v>
       </c>
-      <c r="C66" s="56" t="s">
+      <c r="C66" s="45" t="s">
         <v>623</v>
       </c>
-      <c r="D66" s="56" t="s">
+      <c r="D66" s="45" t="s">
         <v>624</v>
       </c>
       <c r="E66" s="2"/>
@@ -7187,17 +7249,17 @@
       </c>
       <c r="G66" s="4"/>
     </row>
-    <row r="67" spans="1:7" ht="30">
+    <row r="67" spans="1:7" ht="29">
       <c r="A67" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B67" s="4">
         <v>2</v>
       </c>
-      <c r="C67" s="56" t="s">
+      <c r="C67" s="45" t="s">
         <v>622</v>
       </c>
-      <c r="D67" s="56" t="s">
+      <c r="D67" s="45" t="s">
         <v>625</v>
       </c>
       <c r="E67" s="2"/>
@@ -7225,17 +7287,17 @@
       </c>
       <c r="G68" s="4"/>
     </row>
-    <row r="69" spans="1:7" ht="45">
+    <row r="69" spans="1:7" ht="43.5">
       <c r="A69" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B69" s="4">
         <v>4</v>
       </c>
-      <c r="C69" s="56" t="s">
+      <c r="C69" s="45" t="s">
         <v>621</v>
       </c>
-      <c r="D69" s="56" t="s">
+      <c r="D69" s="45" t="s">
         <v>626</v>
       </c>
       <c r="E69" s="2"/>
@@ -7244,17 +7306,17 @@
       </c>
       <c r="G69" s="4"/>
     </row>
-    <row r="70" spans="1:7" ht="30">
+    <row r="70" spans="1:7" ht="29">
       <c r="A70" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B70" s="4">
         <v>5</v>
       </c>
-      <c r="C70" s="56" t="s">
+      <c r="C70" s="45" t="s">
         <v>617</v>
       </c>
-      <c r="D70" s="56" t="s">
+      <c r="D70" s="45" t="s">
         <v>618</v>
       </c>
       <c r="E70" s="2"/>
@@ -7282,17 +7344,17 @@
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:7" ht="30">
+    <row r="72" spans="1:7" ht="29">
       <c r="A72" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B72" s="4">
         <v>7</v>
       </c>
-      <c r="C72" s="56" t="s">
+      <c r="C72" s="45" t="s">
         <v>616</v>
       </c>
-      <c r="D72" s="56" t="s">
+      <c r="D72" s="45" t="s">
         <v>619</v>
       </c>
       <c r="E72" s="2"/>
@@ -7301,17 +7363,17 @@
       </c>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:7" ht="30">
+    <row r="73" spans="1:7" ht="29">
       <c r="A73" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B73" s="4">
         <v>8</v>
       </c>
-      <c r="C73" s="56" t="s">
+      <c r="C73" s="45" t="s">
         <v>615</v>
       </c>
-      <c r="D73" s="56" t="s">
+      <c r="D73" s="45" t="s">
         <v>620</v>
       </c>
       <c r="E73" s="2"/>
@@ -7339,17 +7401,17 @@
       </c>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:7" ht="30">
+    <row r="75" spans="1:7" ht="29">
       <c r="A75" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B75" s="4">
         <v>10</v>
       </c>
-      <c r="C75" s="56" t="s">
+      <c r="C75" s="45" t="s">
         <v>609</v>
       </c>
-      <c r="D75" s="56" t="s">
+      <c r="D75" s="45" t="s">
         <v>612</v>
       </c>
       <c r="E75" s="2"/>
@@ -7358,17 +7420,17 @@
       </c>
       <c r="G75" s="4"/>
     </row>
-    <row r="76" spans="1:7" ht="30">
+    <row r="76" spans="1:7" ht="29">
       <c r="A76" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B76" s="4">
         <v>11</v>
       </c>
-      <c r="C76" s="56" t="s">
+      <c r="C76" s="45" t="s">
         <v>610</v>
       </c>
-      <c r="D76" s="56" t="s">
+      <c r="D76" s="45" t="s">
         <v>613</v>
       </c>
       <c r="E76" s="2"/>
@@ -7377,17 +7439,17 @@
       </c>
       <c r="G76" s="4"/>
     </row>
-    <row r="77" spans="1:7" ht="30">
+    <row r="77" spans="1:7" ht="29">
       <c r="A77" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B77" s="4">
         <v>12</v>
       </c>
-      <c r="C77" s="56" t="s">
+      <c r="C77" s="45" t="s">
         <v>611</v>
       </c>
-      <c r="D77" s="56" t="s">
+      <c r="D77" s="45" t="s">
         <v>614</v>
       </c>
       <c r="E77" s="2"/>
@@ -7453,17 +7515,17 @@
       </c>
       <c r="G80" s="4"/>
     </row>
-    <row r="81" spans="1:7" ht="30">
+    <row r="81" spans="1:7" ht="29">
       <c r="A81" s="2" t="s">
         <v>560</v>
       </c>
       <c r="B81" s="4">
         <v>16</v>
       </c>
-      <c r="C81" s="56" t="s">
+      <c r="C81" s="45" t="s">
         <v>607</v>
       </c>
-      <c r="D81" s="56" t="s">
+      <c r="D81" s="45" t="s">
         <v>608</v>
       </c>
       <c r="E81" s="2"/>
@@ -7927,6 +7989,40 @@
         <v>8</v>
       </c>
       <c r="G105" s="4"/>
+    </row>
+    <row r="106" spans="1:7">
+      <c r="A106" s="59" t="s">
+        <v>627</v>
+      </c>
+      <c r="B106" s="4">
+        <v>1</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="E106" s="2"/>
+      <c r="F106" s="4"/>
+      <c r="G106" s="4"/>
+    </row>
+    <row r="107" spans="1:7">
+      <c r="A107" s="59" t="s">
+        <v>627</v>
+      </c>
+      <c r="B107" s="4">
+        <v>2</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="E107" s="2"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
@@ -7937,14 +8033,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="18" customHeight="1">
@@ -7986,7 +8082,7 @@
       </c>
       <c r="C2" t="str">
         <f ca="1">TEXT(YEAR(NOW())-2000,"00")&amp;TEXT(MONTH(NOW()),"00")&amp;TEXT(DAY(NOW()),"00")&amp;TEXT(HOUR(NOW()),"00")&amp;TEXT(MINUTE(NOW()),"00")</f>
-        <v>2608101435</v>
+        <v>2608120812</v>
       </c>
       <c r="F2" t="s">
         <v>104</v>
@@ -8000,27 +8096,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Q1000"/>
-  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="12.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="7" width="41.140625" customWidth="1"/>
-    <col min="8" max="17" width="12.5703125" customWidth="1"/>
+    <col min="1" max="7" width="41.1796875" customWidth="1"/>
+    <col min="8" max="17" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75">
-      <c r="A1" s="44" t="s">
+    <row r="1" spans="1:17" ht="15.5">
+      <c r="A1" s="46" t="s">
         <v>307</v>
       </c>
-      <c r="B1" s="45"/>
+      <c r="B1" s="47"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="47"/>
+      <c r="A2" s="48"/>
+      <c r="B2" s="49"/>
     </row>
     <row r="3" spans="1:17" ht="99" customHeight="1">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="50" t="s">
         <v>312</v>
       </c>
-      <c r="B3" s="49"/>
+      <c r="B3" s="51"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="5" spans="1:17" ht="18" customHeight="1">
@@ -9096,28 +9192,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AD1000"/>
-  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="12.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="30" width="41.140625" customWidth="1"/>
+    <col min="1" max="30" width="41.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15.75">
-      <c r="A1" s="44" t="s">
+    <row r="1" spans="1:30" ht="15.5">
+      <c r="A1" s="46" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="45"/>
+      <c r="B1" s="47"/>
       <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="47"/>
+      <c r="A2" s="48"/>
+      <c r="B2" s="49"/>
       <c r="C2" s="18"/>
     </row>
     <row r="3" spans="1:30" ht="96.75" customHeight="1">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="50" t="s">
         <v>320</v>
       </c>
-      <c r="B3" s="49"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="18"/>
     </row>
     <row r="4" spans="1:30" ht="15.75" customHeight="1">
@@ -9311,10 +9407,10 @@
       <c r="C7" s="18"/>
     </row>
     <row r="8" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="52" t="s">
         <v>347</v>
       </c>
-      <c r="B8" s="51"/>
+      <c r="B8" s="53"/>
       <c r="C8" s="22"/>
       <c r="D8" s="23"/>
       <c r="E8" s="23"/>
@@ -11835,10 +11931,10 @@
       <c r="C75" s="18"/>
     </row>
     <row r="76" spans="1:30" ht="15.75" customHeight="1">
-      <c r="A76" s="52" t="s">
+      <c r="A76" s="54" t="s">
         <v>199</v>
       </c>
-      <c r="B76" s="51"/>
+      <c r="B76" s="53"/>
       <c r="C76" s="28"/>
       <c r="D76" s="29"/>
       <c r="E76" s="30"/>
@@ -13390,35 +13486,35 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:P1000"/>
-  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="12.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="6" width="41.140625" customWidth="1"/>
-    <col min="7" max="16" width="12.5703125" customWidth="1"/>
+    <col min="1" max="6" width="41.1796875" customWidth="1"/>
+    <col min="7" max="16" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="55" t="s">
         <v>309</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="56"/>
       <c r="C1" s="37"/>
       <c r="D1" s="37"/>
       <c r="E1" s="37"/>
       <c r="F1" s="37"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="47"/>
+      <c r="A2" s="48"/>
+      <c r="B2" s="49"/>
       <c r="C2" s="37"/>
       <c r="D2" s="37"/>
       <c r="E2" s="37"/>
       <c r="F2" s="37"/>
     </row>
     <row r="3" spans="1:16" ht="54.75" customHeight="1">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="50" t="s">
         <v>310</v>
       </c>
-      <c r="B3" s="49"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="37"/>
       <c r="D3" s="37"/>
       <c r="E3" s="37"/>

</xml_diff>